<commit_message>
Split labelling tool into per-country sheets; fix AFG column name
- Read update_survey per country (sheet = country_assessment) instead
  of one shared "update_survey" sheet, now that
  edu_indicator_labelling.xlsx has a dedicated sheet per country.
- Fix AFG's add_cols_tot to pull "child_school_type" instead of
  "children_schooling_type" (regenerates input_tool/03_loa/loa_analysis_AFG.csv
  accordingly).
- Drop the "_orig" suffix from the labeled_results_table debug CSV filename.
- Normalize string quoting (single -> double) across touched files; no
  functional change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015BPqN4aYg38KYgSBbxDEJR
</commit_message>
<xml_diff>
--- a/input_tool/edu_indicator_labelling.xlsx
+++ b/input_tool/edu_indicator_labelling.xlsx
@@ -8,32 +8,34 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\EduAnalysisTool-v2-worktrees\main-config-validation\input_tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F60E814B-3F92-4257-AA15-BA7E71F58FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAF8901-9C36-4FC6-B9A1-00D39C4DEF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1245" yWindow="-15870" windowWidth="25440" windowHeight="15990" tabRatio="834" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="834" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="update_survey" sheetId="6" r:id="rId1"/>
     <sheet name="original" sheetId="22" r:id="rId2"/>
-    <sheet name="bfa" sheetId="21" r:id="rId3"/>
-    <sheet name="lbn" sheetId="20" r:id="rId4"/>
-    <sheet name="hti" sheetId="19" r:id="rId5"/>
-    <sheet name="eth" sheetId="18" r:id="rId6"/>
-    <sheet name="drc" sheetId="17" r:id="rId7"/>
-    <sheet name="ssd" sheetId="16" r:id="rId8"/>
-    <sheet name="som" sheetId="15" r:id="rId9"/>
-    <sheet name="mmr" sheetId="14" r:id="rId10"/>
-    <sheet name="mali" sheetId="13" r:id="rId11"/>
-    <sheet name="ken" sheetId="12" r:id="rId12"/>
-    <sheet name="moz" sheetId="11" r:id="rId13"/>
-    <sheet name="update_choices" sheetId="7" r:id="rId14"/>
-    <sheet name="car" sheetId="8" r:id="rId15"/>
-    <sheet name="afg" sheetId="9" r:id="rId16"/>
-    <sheet name="sdn" sheetId="10" r:id="rId17"/>
+    <sheet name="update_choices" sheetId="7" r:id="rId3"/>
+    <sheet name="OPT" sheetId="23" r:id="rId4"/>
+    <sheet name="BFA" sheetId="21" r:id="rId5"/>
+    <sheet name="LBN" sheetId="20" r:id="rId6"/>
+    <sheet name="HTI" sheetId="19" r:id="rId7"/>
+    <sheet name="ETH" sheetId="18" r:id="rId8"/>
+    <sheet name="DRC" sheetId="17" r:id="rId9"/>
+    <sheet name="SSD" sheetId="16" r:id="rId10"/>
+    <sheet name="SOM" sheetId="15" r:id="rId11"/>
+    <sheet name="MMR" sheetId="14" r:id="rId12"/>
+    <sheet name="MLI" sheetId="13" r:id="rId13"/>
+    <sheet name="KEN" sheetId="12" r:id="rId14"/>
+    <sheet name="MOZ" sheetId="11" r:id="rId15"/>
+    <sheet name="CAR" sheetId="8" r:id="rId16"/>
+    <sheet name="AFG" sheetId="9" r:id="rId17"/>
+    <sheet name="SDN" sheetId="10" r:id="rId18"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">OPT!#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">original!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">update_choices!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">update_choices!$A$1:$H$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">update_survey!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -60,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3186" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3376" uniqueCount="237">
   <si>
     <t>theme</t>
   </si>
@@ -1723,7 +1725,7 @@
       </c>
       <c r="F24" s="26"/>
     </row>
-    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" ht="36" x14ac:dyDescent="0.4">
       <c r="A25" s="7" t="s">
         <v>1</v>
       </c>
@@ -1740,7 +1742,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" ht="36" x14ac:dyDescent="0.4">
       <c r="A26" s="7" t="s">
         <v>1</v>
       </c>
@@ -1980,11 +1982,12 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBB2A30-1E77-42F1-964E-A72E9BDDBED9}">
-  <dimension ref="A1:F39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C98E618-344A-487D-B00E-EFB2C24E3770}">
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="53.5" style="7"/>
+    <col min="1" max="1" width="19.19921875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="16.3984375" style="7" customWidth="1"/>
     <col min="3" max="5" width="53.5" style="15"/>
     <col min="6" max="16384" width="53.5" style="7"/>
   </cols>
@@ -2206,7 +2209,7 @@
         <v>169</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>42</v>
+        <v>209</v>
       </c>
       <c r="E13" s="17" t="s">
         <v>49</v>
@@ -2380,7 +2383,7 @@
         <v>31</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E23" s="26" t="s">
         <v>197</v>
@@ -2643,6 +2646,23 @@
       </c>
       <c r="D39" s="15" t="s">
         <v>175</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -2661,7 +2681,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FDAFB7B-CACC-4A95-AEE0-FBF416C1C9E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BA04313-1E16-4C5B-AB02-8927EAB717AE}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
   <cols>
@@ -2887,7 +2907,7 @@
         <v>169</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>42</v>
+        <v>209</v>
       </c>
       <c r="E13" s="17" t="s">
         <v>49</v>
@@ -2907,7 +2927,7 @@
         <v>43</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>202</v>
+        <v>47</v>
       </c>
       <c r="F14" s="26"/>
     </row>
@@ -2922,10 +2942,10 @@
         <v>27</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>203</v>
+        <v>230</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>49</v>
       </c>
       <c r="F15" s="28"/>
     </row>
@@ -2940,10 +2960,10 @@
         <v>28</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>233</v>
+        <v>225</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>48</v>
       </c>
       <c r="F16" s="28"/>
     </row>
@@ -3046,7 +3066,7 @@
         <v>106</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="F22" s="26"/>
     </row>
@@ -3061,10 +3081,10 @@
         <v>31</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="F23" s="26"/>
     </row>
@@ -3079,10 +3099,10 @@
         <v>167</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="F24" s="26"/>
     </row>
@@ -3342,7 +3362,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C9AFB8-F0F3-4AAA-AA27-0292EA78AA26}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBB2A30-1E77-42F1-964E-A72E9BDDBED9}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
   <cols>
@@ -3603,7 +3623,7 @@
         <v>27</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>199</v>
+        <v>230</v>
       </c>
       <c r="E15" s="27" t="s">
         <v>49</v>
@@ -3621,7 +3641,7 @@
         <v>28</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="E16" s="27" t="s">
         <v>48</v>
@@ -3742,7 +3762,7 @@
         <v>31</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E23" s="26" t="s">
         <v>197</v>
@@ -3760,7 +3780,7 @@
         <v>167</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="E24" s="26" t="s">
         <v>198</v>
@@ -4023,7 +4043,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD3426F2-D478-46D5-B931-E2053F6BF542}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FDAFB7B-CACC-4A95-AEE0-FBF416C1C9E5}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
   <cols>
@@ -4269,7 +4289,7 @@
         <v>43</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>47</v>
+        <v>202</v>
       </c>
       <c r="F14" s="26"/>
     </row>
@@ -4284,10 +4304,10 @@
         <v>27</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>49</v>
+        <v>199</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>203</v>
       </c>
       <c r="F15" s="28"/>
     </row>
@@ -4302,10 +4322,10 @@
         <v>28</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>48</v>
+        <v>232</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>233</v>
       </c>
       <c r="F16" s="28"/>
     </row>
@@ -4408,7 +4428,7 @@
         <v>106</v>
       </c>
       <c r="E22" s="26" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="F22" s="26"/>
     </row>
@@ -4423,10 +4443,10 @@
         <v>31</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="E23" s="26" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="F23" s="26"/>
     </row>
@@ -4441,10 +4461,10 @@
         <v>167</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="E24" s="26" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F24" s="26"/>
     </row>
@@ -4704,472 +4724,1368 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C9AFB8-F0F3-4AAA-AA27-0292EA78AA26}">
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="36.09765625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="54.3984375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.3984375" style="1" customWidth="1"/>
-    <col min="5" max="8" width="12.69921875" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="1"/>
+    <col min="1" max="2" width="53.5" style="7"/>
+    <col min="3" max="5" width="53.5" style="15"/>
+    <col min="6" max="16384" width="53.5" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A9" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A12" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A19" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A20" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A21" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A22" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A25" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A26" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A28" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A29" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A30" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A31" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>140</v>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A5" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A7" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A9" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="26"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="26"/>
+    </row>
+    <row r="12" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A12" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A13" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="26"/>
+    </row>
+    <row r="15" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A15" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="28"/>
+    </row>
+    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A16" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="28"/>
+    </row>
+    <row r="17" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A17" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A18" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A19" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F22" s="26"/>
+    </row>
+    <row r="23" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="F23" s="26"/>
+    </row>
+    <row r="24" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="F24" s="26"/>
+    </row>
+    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+      <c r="A25" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+      <c r="A26" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A31" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A32" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H19" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <mergeCells count="8">
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E22:F22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD3426F2-D478-46D5-B931-E2053F6BF542}">
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="2" width="53.5" style="7"/>
+    <col min="3" max="5" width="53.5" style="15"/>
+    <col min="6" max="16384" width="53.5" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A5" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A7" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A9" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="26"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="26"/>
+    </row>
+    <row r="12" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A12" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A13" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="26"/>
+    </row>
+    <row r="15" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A15" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="28"/>
+    </row>
+    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A16" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="28"/>
+    </row>
+    <row r="17" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A17" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A18" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A19" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F22" s="26"/>
+    </row>
+    <row r="23" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="F23" s="26"/>
+    </row>
+    <row r="24" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="F24" s="26"/>
+    </row>
+    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+      <c r="A25" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+      <c r="A26" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A31" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A32" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E22:F22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F93BDC91-E487-4F88-AEAB-B2FA5E4CA8B4}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -5851,7 +6767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04631CBF-6FD9-45D1-9C42-22D5C9F097A4}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -6533,7 +7449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E3B9F7-D347-4317-AB67-0217058F4008}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -7649,7 +8565,7 @@
       </c>
       <c r="F24" s="26"/>
     </row>
-    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:6" ht="36" x14ac:dyDescent="0.4">
       <c r="A25" s="7" t="s">
         <v>1</v>
       </c>
@@ -7666,7 +8582,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:6" ht="36" x14ac:dyDescent="0.4">
       <c r="A26" s="7" t="s">
         <v>1</v>
       </c>
@@ -7906,6 +8822,1157 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="36.09765625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="54.3984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.3984375" style="1" customWidth="1"/>
+    <col min="5" max="8" width="12.69921875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A22" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A23" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A25" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A26" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A28" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A29" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A30" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A31" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H19" xr:uid="{00000000-0001-0000-0600-000000000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E37EE543-B5CB-4185-B91B-2A9A8CC3DA4C}">
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="24.5" style="7" customWidth="1"/>
+    <col min="2" max="2" width="26.59765625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="53.5" style="15"/>
+    <col min="4" max="4" width="106.5" style="15" customWidth="1"/>
+    <col min="5" max="5" width="53.5" style="15"/>
+    <col min="6" max="16384" width="53.5" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A5" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A7" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A8" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A9" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A10" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="26"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="26"/>
+    </row>
+    <row r="12" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A12" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A13" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="26"/>
+    </row>
+    <row r="15" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A15" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="28"/>
+    </row>
+    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A16" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="28"/>
+    </row>
+    <row r="17" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A17" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A18" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A19" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
+      <c r="A20" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F22" s="26"/>
+    </row>
+    <row r="23" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="F23" s="26"/>
+    </row>
+    <row r="24" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="F24" s="26"/>
+    </row>
+    <row r="25" spans="1:6" ht="36" x14ac:dyDescent="0.4">
+      <c r="A25" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="36" x14ac:dyDescent="0.4">
+      <c r="A26" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A29" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A30" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A31" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A32" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E22:F22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78ED0E70-DB3B-451B-8866-F48A2CB32CE9}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -8587,7 +10654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B023821-20D2-4192-846D-05966B68C2F4}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -9269,7 +11336,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E598F01-CD75-4BC5-AD14-CB9738585B67}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -9951,7 +12018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{664A1F51-322B-4DAC-988D-ED5F1BCA03D1}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -10638,7 +12705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1430A0F1-2F5D-43E5-9E49-8E679EDD81F4}">
   <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
@@ -11323,1384 +13390,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C98E618-344A-487D-B00E-EFB2C24E3770}">
-  <dimension ref="A1:F40"/>
-  <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="1" width="19.19921875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="16.3984375" style="7" customWidth="1"/>
-    <col min="3" max="5" width="53.5" style="15"/>
-    <col min="6" max="16384" width="53.5" style="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A7" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A8" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A9" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="26"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="26"/>
-    </row>
-    <row r="12" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A12" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A13" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="26"/>
-    </row>
-    <row r="15" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A15" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="28"/>
-    </row>
-    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A16" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="28"/>
-    </row>
-    <row r="17" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A17" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A18" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A19" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A20" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A21" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="F22" s="26"/>
-    </row>
-    <row r="23" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>210</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="F23" s="26"/>
-    </row>
-    <row r="24" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>167</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="E24" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="F24" s="26"/>
-    </row>
-    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
-      <c r="A25" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>220</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
-      <c r="A26" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A27" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A29" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A30" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A31" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A32" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A34" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>153</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="C40" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="D40" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="E40" s="15" t="s">
-        <v>219</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E22:F22"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BA04313-1E16-4C5B-AB02-8927EAB717AE}">
-  <dimension ref="A1:F39"/>
-  <sheetFormatPr defaultColWidth="53.5" defaultRowHeight="19.2" x14ac:dyDescent="0.4"/>
-  <cols>
-    <col min="1" max="2" width="53.5" style="7"/>
-    <col min="3" max="5" width="53.5" style="15"/>
-    <col min="6" max="16384" width="53.5" style="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>223</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A7" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A8" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A9" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="26"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="26"/>
-    </row>
-    <row r="12" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A12" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A13" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="26"/>
-    </row>
-    <row r="15" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A15" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>230</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="28"/>
-    </row>
-    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A16" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="28"/>
-    </row>
-    <row r="17" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A17" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A18" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A19" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="12" customFormat="1" ht="18" x14ac:dyDescent="0.4">
-      <c r="A20" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A21" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>218</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="F22" s="26"/>
-    </row>
-    <row r="23" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>210</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="F23" s="26"/>
-    </row>
-    <row r="24" spans="1:6" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>167</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="E24" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="F24" s="26"/>
-    </row>
-    <row r="25" spans="1:6" ht="54" x14ac:dyDescent="0.4">
-      <c r="A25" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>220</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="54" x14ac:dyDescent="0.4">
-      <c r="A26" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A27" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A28" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A29" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A30" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>229</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A31" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A32" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="E32" s="15" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A34" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>153</v>
-      </c>
-      <c r="E34" s="15" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="D38" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="E22:F22"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>